<commit_message>
Update Appium runner with verified Samsung SM-A356E device metadata (UDID RZCY60BXV0K)
</commit_message>
<xml_diff>
--- a/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
+++ b/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>AI Assistant</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -644,14 +644,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Pet Sitter</t>
+          <t>Pet Owner</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -686,7 +686,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>QR &amp; Security</t>
+          <t>Forms Validation</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -707,14 +707,14 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>QR &amp; Security</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0</v>
@@ -728,14 +728,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Forms Validation</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -749,14 +749,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Pet Owner</t>
+          <t>Pet Sitter</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:14:56</t>
+          <t>2026-07-29 02:18:41</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Execute Appium mobile test suite on Samsung SM-A356E device and generate HTML & Excel reports
</commit_message>
<xml_diff>
--- a/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
+++ b/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
     </row>
@@ -623,14 +623,14 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0</v>
@@ -644,14 +644,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Pet Owner</t>
+          <t>QR &amp; Security</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>AI Assistant</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -686,7 +686,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Forms Validation</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -707,7 +707,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>QR &amp; Security</t>
+          <t>Forms Validation</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -728,14 +728,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Pet Sitter</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -749,14 +749,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Pet Sitter</t>
+          <t>Pet Owner</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:18:41</t>
+          <t>2026-07-29 02:20:46</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Execute Appium mobile test suite on physical Samsung SM-A356E device with active server and capture screenshots
</commit_message>
<xml_diff>
--- a/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
+++ b/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:13</t>
         </is>
       </c>
     </row>
@@ -623,14 +623,14 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0</v>
@@ -644,14 +644,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>QR &amp; Security</t>
+          <t>Pet Sitter</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant</t>
+          <t>QR &amp; Security</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -686,7 +686,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Forms Validation</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -707,14 +707,14 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Forms Validation</t>
+          <t>Pet Owner</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0</v>
@@ -728,14 +728,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Pet Sitter</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -749,14 +749,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Pet Owner</t>
+          <t>AI Assistant</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -867,7 +867,7 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:00</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:00</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:01</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:01</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:02</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:02</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:03</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:03</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:04</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:05</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:05</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:06</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:06</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1387,7 +1387,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:07</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:08</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:08</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:09</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:10</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:10</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:11</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:12</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:12</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:20:46</t>
+          <t>2026-07-29 02:33:13</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Disable screenshot capture in Appium test suite and update clean HTML/Excel reports
</commit_message>
<xml_diff>
--- a/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
+++ b/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:16</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>QR &amp; Security</t>
+          <t>UI/UX &amp; Edge Cases</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -644,14 +644,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>UI/UX &amp; Edge Cases</t>
+          <t>AI Assistant</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -686,14 +686,14 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Pet Sitter Profile</t>
+          <t>QR &amp; Security</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>0</v>
@@ -728,14 +728,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant</t>
+          <t>Pet Owner Profile</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -749,14 +749,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Pet Owner Profile</t>
+          <t>Pet Sitter Profile</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -863,11 +863,11 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -903,11 +903,11 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -983,11 +983,11 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1063,11 +1063,11 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1103,11 +1103,11 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:43</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1143,11 +1143,11 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:44</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1183,11 +1183,11 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:44</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1223,11 +1223,11 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:44</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1263,11 +1263,11 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1343,11 +1343,11 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1383,11 +1383,11 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1423,11 +1423,11 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1463,11 +1463,11 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1503,11 +1503,11 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1543,11 +1543,11 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1583,11 +1583,11 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1663,11 +1663,11 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:45</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1703,11 +1703,11 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1783,11 +1783,11 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1823,11 +1823,11 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1863,11 +1863,11 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1903,11 +1903,11 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:46</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1943,11 +1943,11 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1983,11 +1983,11 @@
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2023,11 +2023,11 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2063,11 +2063,11 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2103,11 +2103,11 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2143,11 +2143,11 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2183,11 +2183,11 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2263,11 +2263,11 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2303,11 +2303,11 @@
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2343,11 +2343,11 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2383,11 +2383,11 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:47</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2423,11 +2423,11 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2463,11 +2463,11 @@
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2503,11 +2503,11 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2543,11 +2543,11 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2583,11 +2583,11 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -2623,11 +2623,11 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -2663,11 +2663,11 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -2703,11 +2703,11 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -2743,11 +2743,11 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -2783,11 +2783,11 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -2823,11 +2823,11 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -2863,11 +2863,11 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
@@ -2903,11 +2903,11 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -2943,11 +2943,11 @@
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -2983,11 +2983,11 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:48</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -3023,11 +3023,11 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -3063,11 +3063,11 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -3103,11 +3103,11 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
@@ -3143,11 +3143,11 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -3183,11 +3183,11 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
@@ -3223,11 +3223,11 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:49</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
@@ -3263,11 +3263,11 @@
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:50</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -3303,11 +3303,11 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:50</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -3343,11 +3343,11 @@
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:51</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
@@ -3383,11 +3383,11 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -3423,11 +3423,11 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -3463,11 +3463,11 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -3503,11 +3503,11 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -3543,11 +3543,11 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -3583,11 +3583,11 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -3623,11 +3623,11 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
@@ -3663,11 +3663,11 @@
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -3743,11 +3743,11 @@
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
@@ -3783,11 +3783,11 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -3823,11 +3823,11 @@
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -3863,11 +3863,11 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:52</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -3903,11 +3903,11 @@
         </is>
       </c>
       <c r="F78" s="4" t="n">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:53</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -3943,11 +3943,11 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:53</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -3983,11 +3983,11 @@
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:53</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -4023,11 +4023,11 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -4063,11 +4063,11 @@
         </is>
       </c>
       <c r="F82" s="4" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -4103,11 +4103,11 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -4143,11 +4143,11 @@
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
@@ -4183,11 +4183,11 @@
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
@@ -4223,11 +4223,11 @@
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
@@ -4263,11 +4263,11 @@
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -4303,11 +4303,11 @@
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
@@ -4343,11 +4343,11 @@
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -4383,11 +4383,11 @@
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -4423,11 +4423,11 @@
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
@@ -4463,11 +4463,11 @@
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
@@ -4503,11 +4503,11 @@
         </is>
       </c>
       <c r="F93" s="4" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -4543,11 +4543,11 @@
         </is>
       </c>
       <c r="F94" s="4" t="n">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
@@ -4583,11 +4583,11 @@
         </is>
       </c>
       <c r="F95" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
@@ -4623,11 +4623,11 @@
         </is>
       </c>
       <c r="F96" s="4" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
@@ -4663,11 +4663,11 @@
         </is>
       </c>
       <c r="F97" s="4" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:54</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr">
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="F98" s="4" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr">
@@ -4743,11 +4743,11 @@
         </is>
       </c>
       <c r="F99" s="4" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
@@ -4783,11 +4783,11 @@
         </is>
       </c>
       <c r="F100" s="4" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
@@ -4823,11 +4823,11 @@
         </is>
       </c>
       <c r="F101" s="4" t="n">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
@@ -4863,11 +4863,11 @@
         </is>
       </c>
       <c r="F102" s="4" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
@@ -4903,11 +4903,11 @@
         </is>
       </c>
       <c r="F103" s="4" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr">
@@ -4943,11 +4943,11 @@
         </is>
       </c>
       <c r="F104" s="4" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H104" s="4" t="inlineStr">
@@ -4983,11 +4983,11 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -5023,11 +5023,11 @@
         </is>
       </c>
       <c r="F106" s="4" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
@@ -5063,11 +5063,11 @@
         </is>
       </c>
       <c r="F107" s="4" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
@@ -5103,11 +5103,11 @@
         </is>
       </c>
       <c r="F108" s="4" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:55</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
@@ -5143,11 +5143,11 @@
         </is>
       </c>
       <c r="F109" s="4" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
@@ -5183,11 +5183,11 @@
         </is>
       </c>
       <c r="F110" s="4" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
@@ -5223,11 +5223,11 @@
         </is>
       </c>
       <c r="F111" s="4" t="n">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr">
@@ -5263,11 +5263,11 @@
         </is>
       </c>
       <c r="F112" s="4" t="n">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H112" s="4" t="inlineStr">
@@ -5303,11 +5303,11 @@
         </is>
       </c>
       <c r="F113" s="4" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr">
@@ -5343,11 +5343,11 @@
         </is>
       </c>
       <c r="F114" s="4" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H114" s="4" t="inlineStr">
@@ -5383,11 +5383,11 @@
         </is>
       </c>
       <c r="F115" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H115" s="4" t="inlineStr">
@@ -5423,11 +5423,11 @@
         </is>
       </c>
       <c r="F116" s="4" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H116" s="4" t="inlineStr">
@@ -5463,11 +5463,11 @@
         </is>
       </c>
       <c r="F117" s="4" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H117" s="4" t="inlineStr">
@@ -5503,11 +5503,11 @@
         </is>
       </c>
       <c r="F118" s="4" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H118" s="4" t="inlineStr">
@@ -5543,11 +5543,11 @@
         </is>
       </c>
       <c r="F119" s="4" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H119" s="4" t="inlineStr">
@@ -5583,11 +5583,11 @@
         </is>
       </c>
       <c r="F120" s="4" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:56</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H120" s="4" t="inlineStr">
@@ -5623,11 +5623,11 @@
         </is>
       </c>
       <c r="F121" s="4" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H121" s="4" t="inlineStr">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="F122" s="4" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="G122" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H122" s="4" t="inlineStr">
@@ -5703,11 +5703,11 @@
         </is>
       </c>
       <c r="F123" s="4" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H123" s="4" t="inlineStr">
@@ -5743,11 +5743,11 @@
         </is>
       </c>
       <c r="F124" s="4" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H124" s="4" t="inlineStr">
@@ -5783,11 +5783,11 @@
         </is>
       </c>
       <c r="F125" s="4" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H125" s="4" t="inlineStr">
@@ -5823,11 +5823,11 @@
         </is>
       </c>
       <c r="F126" s="4" t="n">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="G126" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H126" s="4" t="inlineStr">
@@ -5863,11 +5863,11 @@
         </is>
       </c>
       <c r="F127" s="4" t="n">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H127" s="4" t="inlineStr">
@@ -5903,11 +5903,11 @@
         </is>
       </c>
       <c r="F128" s="4" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G128" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:57</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H128" s="4" t="inlineStr">
@@ -5943,11 +5943,11 @@
         </is>
       </c>
       <c r="F129" s="4" t="n">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H129" s="4" t="inlineStr">
@@ -5983,11 +5983,11 @@
         </is>
       </c>
       <c r="F130" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G130" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H130" s="4" t="inlineStr">
@@ -6023,11 +6023,11 @@
         </is>
       </c>
       <c r="F131" s="4" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G131" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H131" s="4" t="inlineStr">
@@ -6063,11 +6063,11 @@
         </is>
       </c>
       <c r="F132" s="4" t="n">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="G132" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H132" s="4" t="inlineStr">
@@ -6107,7 +6107,7 @@
       </c>
       <c r="G133" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H133" s="4" t="inlineStr">
@@ -6143,11 +6143,11 @@
         </is>
       </c>
       <c r="F134" s="4" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="G134" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H134" s="4" t="inlineStr">
@@ -6183,11 +6183,11 @@
         </is>
       </c>
       <c r="F135" s="4" t="n">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="G135" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:58</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H135" s="4" t="inlineStr">
@@ -6223,11 +6223,11 @@
         </is>
       </c>
       <c r="F136" s="4" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:35:59</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H136" s="4" t="inlineStr">
@@ -6263,11 +6263,11 @@
         </is>
       </c>
       <c r="F137" s="4" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G137" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H137" s="4" t="inlineStr">
@@ -6303,11 +6303,11 @@
         </is>
       </c>
       <c r="F138" s="4" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="G138" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H138" s="4" t="inlineStr">
@@ -6343,11 +6343,11 @@
         </is>
       </c>
       <c r="F139" s="4" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="G139" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H139" s="4" t="inlineStr">
@@ -6383,11 +6383,11 @@
         </is>
       </c>
       <c r="F140" s="4" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G140" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H140" s="4" t="inlineStr">
@@ -6427,7 +6427,7 @@
       </c>
       <c r="G141" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H141" s="4" t="inlineStr">
@@ -6463,11 +6463,11 @@
         </is>
       </c>
       <c r="F142" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G142" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H142" s="4" t="inlineStr">
@@ -6503,11 +6503,11 @@
         </is>
       </c>
       <c r="F143" s="4" t="n">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="G143" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H143" s="4" t="inlineStr">
@@ -6543,11 +6543,11 @@
         </is>
       </c>
       <c r="F144" s="4" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H144" s="4" t="inlineStr">
@@ -6583,11 +6583,11 @@
         </is>
       </c>
       <c r="F145" s="4" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H145" s="4" t="inlineStr">
@@ -6627,7 +6627,7 @@
       </c>
       <c r="G146" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H146" s="4" t="inlineStr">
@@ -6663,11 +6663,11 @@
         </is>
       </c>
       <c r="F147" s="4" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H147" s="4" t="inlineStr">
@@ -6703,11 +6703,11 @@
         </is>
       </c>
       <c r="F148" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr">
@@ -6743,11 +6743,11 @@
         </is>
       </c>
       <c r="F149" s="4" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:00</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr">
@@ -6783,11 +6783,11 @@
         </is>
       </c>
       <c r="F150" s="4" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="G150" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H150" s="4" t="inlineStr">
@@ -6823,11 +6823,11 @@
         </is>
       </c>
       <c r="F151" s="4" t="n">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="G151" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H151" s="4" t="inlineStr">
@@ -6863,11 +6863,11 @@
         </is>
       </c>
       <c r="F152" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G152" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H152" s="4" t="inlineStr">
@@ -6903,11 +6903,11 @@
         </is>
       </c>
       <c r="F153" s="4" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="G153" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H153" s="4" t="inlineStr">
@@ -6943,11 +6943,11 @@
         </is>
       </c>
       <c r="F154" s="4" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="G154" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H154" s="4" t="inlineStr">
@@ -6983,11 +6983,11 @@
         </is>
       </c>
       <c r="F155" s="4" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H155" s="4" t="inlineStr">
@@ -7023,11 +7023,11 @@
         </is>
       </c>
       <c r="F156" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H156" s="4" t="inlineStr">
@@ -7063,11 +7063,11 @@
         </is>
       </c>
       <c r="F157" s="4" t="n">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="G157" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H157" s="4" t="inlineStr">
@@ -7103,11 +7103,11 @@
         </is>
       </c>
       <c r="F158" s="4" t="n">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G158" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H158" s="4" t="inlineStr">
@@ -7143,11 +7143,11 @@
         </is>
       </c>
       <c r="F159" s="4" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H159" s="4" t="inlineStr">
@@ -7183,11 +7183,11 @@
         </is>
       </c>
       <c r="F160" s="4" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G160" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:01</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H160" s="4" t="inlineStr">
@@ -7223,11 +7223,11 @@
         </is>
       </c>
       <c r="F161" s="4" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G161" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H161" s="4" t="inlineStr">
@@ -7263,11 +7263,11 @@
         </is>
       </c>
       <c r="F162" s="4" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G162" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H162" s="4" t="inlineStr">
@@ -7303,11 +7303,11 @@
         </is>
       </c>
       <c r="F163" s="4" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G163" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H163" s="4" t="inlineStr">
@@ -7343,11 +7343,11 @@
         </is>
       </c>
       <c r="F164" s="4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H164" s="4" t="inlineStr">
@@ -7383,11 +7383,11 @@
         </is>
       </c>
       <c r="F165" s="4" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="G165" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H165" s="4" t="inlineStr">
@@ -7423,11 +7423,11 @@
         </is>
       </c>
       <c r="F166" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G166" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H166" s="4" t="inlineStr">
@@ -7463,11 +7463,11 @@
         </is>
       </c>
       <c r="F167" s="4" t="n">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="G167" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H167" s="4" t="inlineStr">
@@ -7503,11 +7503,11 @@
         </is>
       </c>
       <c r="F168" s="4" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H168" s="4" t="inlineStr">
@@ -7543,11 +7543,11 @@
         </is>
       </c>
       <c r="F169" s="4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H169" s="4" t="inlineStr">
@@ -7583,11 +7583,11 @@
         </is>
       </c>
       <c r="F170" s="4" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="G170" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H170" s="4" t="inlineStr">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="F171" s="4" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr">
@@ -7663,11 +7663,11 @@
         </is>
       </c>
       <c r="F172" s="4" t="n">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G172" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:02</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H172" s="4" t="inlineStr">
@@ -7703,11 +7703,11 @@
         </is>
       </c>
       <c r="F173" s="4" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G173" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H173" s="4" t="inlineStr">
@@ -7743,11 +7743,11 @@
         </is>
       </c>
       <c r="F174" s="4" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="G174" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H174" s="4" t="inlineStr">
@@ -7783,11 +7783,11 @@
         </is>
       </c>
       <c r="F175" s="4" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G175" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H175" s="4" t="inlineStr">
@@ -7823,11 +7823,11 @@
         </is>
       </c>
       <c r="F176" s="4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G176" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H176" s="4" t="inlineStr">
@@ -7863,11 +7863,11 @@
         </is>
       </c>
       <c r="F177" s="4" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="G177" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr">
@@ -7903,11 +7903,11 @@
         </is>
       </c>
       <c r="F178" s="4" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="G178" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H178" s="4" t="inlineStr">
@@ -7943,11 +7943,11 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G179" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H179" s="4" t="inlineStr">
@@ -7983,11 +7983,11 @@
         </is>
       </c>
       <c r="F180" s="4" t="n">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="G180" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr">
@@ -8023,11 +8023,11 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G181" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H181" s="4" t="inlineStr">
@@ -8063,11 +8063,11 @@
         </is>
       </c>
       <c r="F182" s="4" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G182" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H182" s="4" t="inlineStr">
@@ -8103,11 +8103,11 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G183" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H183" s="4" t="inlineStr">
@@ -8147,7 +8147,7 @@
       </c>
       <c r="G184" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H184" s="4" t="inlineStr">
@@ -8183,11 +8183,11 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G185" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr">
@@ -8223,11 +8223,11 @@
         </is>
       </c>
       <c r="F186" s="4" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G186" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H186" s="4" t="inlineStr">
@@ -8263,11 +8263,11 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G187" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H187" s="4" t="inlineStr">
@@ -8303,11 +8303,11 @@
         </is>
       </c>
       <c r="F188" s="4" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G188" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H188" s="4" t="inlineStr">
@@ -8343,11 +8343,11 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G189" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H189" s="4" t="inlineStr">
@@ -8383,11 +8383,11 @@
         </is>
       </c>
       <c r="F190" s="4" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="G190" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:03</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H190" s="4" t="inlineStr">
@@ -8423,11 +8423,11 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G191" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H191" s="4" t="inlineStr">
@@ -8463,11 +8463,11 @@
         </is>
       </c>
       <c r="F192" s="4" t="n">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="G192" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H192" s="4" t="inlineStr">
@@ -8503,11 +8503,11 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="G193" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H193" s="4" t="inlineStr">
@@ -8543,11 +8543,11 @@
         </is>
       </c>
       <c r="F194" s="4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H194" s="4" t="inlineStr">
@@ -8583,11 +8583,11 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H195" s="4" t="inlineStr">
@@ -8623,11 +8623,11 @@
         </is>
       </c>
       <c r="F196" s="4" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="G196" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H196" s="4" t="inlineStr">
@@ -8663,11 +8663,11 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G197" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H197" s="4" t="inlineStr">
@@ -8703,11 +8703,11 @@
         </is>
       </c>
       <c r="F198" s="4" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="G198" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H198" s="4" t="inlineStr">
@@ -8743,11 +8743,11 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="G199" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H199" s="4" t="inlineStr">
@@ -8783,11 +8783,11 @@
         </is>
       </c>
       <c r="F200" s="4" t="n">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G200" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H200" s="4" t="inlineStr">
@@ -8823,11 +8823,11 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G201" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:04</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H201" s="4" t="inlineStr">
@@ -8867,7 +8867,7 @@
       </c>
       <c r="G202" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:05</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H202" s="4" t="inlineStr">
@@ -8903,11 +8903,11 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G203" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:05</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H203" s="4" t="inlineStr">
@@ -8943,11 +8943,11 @@
         </is>
       </c>
       <c r="F204" s="4" t="n">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="G204" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:05</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H204" s="4" t="inlineStr">
@@ -8983,11 +8983,11 @@
         </is>
       </c>
       <c r="F205" s="4" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G205" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:05</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H205" s="4" t="inlineStr">
@@ -9023,11 +9023,11 @@
         </is>
       </c>
       <c r="F206" s="4" t="n">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="G206" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H206" s="4" t="inlineStr">
@@ -9063,11 +9063,11 @@
         </is>
       </c>
       <c r="F207" s="4" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="G207" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H207" s="4" t="inlineStr">
@@ -9103,11 +9103,11 @@
         </is>
       </c>
       <c r="F208" s="4" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="G208" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H208" s="4" t="inlineStr">
@@ -9143,11 +9143,11 @@
         </is>
       </c>
       <c r="F209" s="4" t="n">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="G209" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H209" s="4" t="inlineStr">
@@ -9183,11 +9183,11 @@
         </is>
       </c>
       <c r="F210" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G210" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H210" s="4" t="inlineStr">
@@ -9223,11 +9223,11 @@
         </is>
       </c>
       <c r="F211" s="4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G211" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H211" s="4" t="inlineStr">
@@ -9263,11 +9263,11 @@
         </is>
       </c>
       <c r="F212" s="4" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G212" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H212" s="4" t="inlineStr">
@@ -9303,11 +9303,11 @@
         </is>
       </c>
       <c r="F213" s="4" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G213" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H213" s="4" t="inlineStr">
@@ -9343,11 +9343,11 @@
         </is>
       </c>
       <c r="F214" s="4" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="G214" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H214" s="4" t="inlineStr">
@@ -9383,11 +9383,11 @@
         </is>
       </c>
       <c r="F215" s="4" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="G215" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H215" s="4" t="inlineStr">
@@ -9423,11 +9423,11 @@
         </is>
       </c>
       <c r="F216" s="4" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G216" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H216" s="4" t="inlineStr">
@@ -9463,11 +9463,11 @@
         </is>
       </c>
       <c r="F217" s="4" t="n">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G217" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H217" s="4" t="inlineStr">
@@ -9503,11 +9503,11 @@
         </is>
       </c>
       <c r="F218" s="4" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G218" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H218" s="4" t="inlineStr">
@@ -9543,11 +9543,11 @@
         </is>
       </c>
       <c r="F219" s="4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G219" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H219" s="4" t="inlineStr">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="F220" s="4" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="G220" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:06</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr">
@@ -9623,11 +9623,11 @@
         </is>
       </c>
       <c r="F221" s="4" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="G221" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H221" s="4" t="inlineStr">
@@ -9663,11 +9663,11 @@
         </is>
       </c>
       <c r="F222" s="4" t="n">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="G222" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H222" s="4" t="inlineStr">
@@ -9703,11 +9703,11 @@
         </is>
       </c>
       <c r="F223" s="4" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr">
@@ -9743,11 +9743,11 @@
         </is>
       </c>
       <c r="F224" s="4" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G224" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H224" s="4" t="inlineStr">
@@ -9783,11 +9783,11 @@
         </is>
       </c>
       <c r="F225" s="4" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="G225" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H225" s="4" t="inlineStr">
@@ -9823,11 +9823,11 @@
         </is>
       </c>
       <c r="F226" s="4" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G226" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H226" s="4" t="inlineStr">
@@ -9863,11 +9863,11 @@
         </is>
       </c>
       <c r="F227" s="4" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="G227" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H227" s="4" t="inlineStr">
@@ -9903,11 +9903,11 @@
         </is>
       </c>
       <c r="F228" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G228" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H228" s="4" t="inlineStr">
@@ -9943,11 +9943,11 @@
         </is>
       </c>
       <c r="F229" s="4" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G229" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H229" s="4" t="inlineStr">
@@ -9983,11 +9983,11 @@
         </is>
       </c>
       <c r="F230" s="4" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="G230" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H230" s="4" t="inlineStr">
@@ -10023,11 +10023,11 @@
         </is>
       </c>
       <c r="F231" s="4" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G231" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H231" s="4" t="inlineStr">
@@ -10063,11 +10063,11 @@
         </is>
       </c>
       <c r="F232" s="4" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G232" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H232" s="4" t="inlineStr">
@@ -10103,11 +10103,11 @@
         </is>
       </c>
       <c r="F233" s="4" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G233" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H233" s="4" t="inlineStr">
@@ -10143,11 +10143,11 @@
         </is>
       </c>
       <c r="F234" s="4" t="n">
-        <v>16</v>
+        <v>43</v>
       </c>
       <c r="G234" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H234" s="4" t="inlineStr">
@@ -10183,11 +10183,11 @@
         </is>
       </c>
       <c r="F235" s="4" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="G235" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:07</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H235" s="4" t="inlineStr">
@@ -10223,11 +10223,11 @@
         </is>
       </c>
       <c r="F236" s="4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G236" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:08</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H236" s="4" t="inlineStr">
@@ -10263,11 +10263,11 @@
         </is>
       </c>
       <c r="F237" s="4" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="G237" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:08</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H237" s="4" t="inlineStr">
@@ -10303,11 +10303,11 @@
         </is>
       </c>
       <c r="F238" s="4" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="G238" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:08</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H238" s="4" t="inlineStr">
@@ -10343,11 +10343,11 @@
         </is>
       </c>
       <c r="F239" s="4" t="n">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="G239" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:08</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H239" s="4" t="inlineStr">
@@ -10383,11 +10383,11 @@
         </is>
       </c>
       <c r="F240" s="4" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="G240" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:08</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H240" s="4" t="inlineStr">
@@ -10423,11 +10423,11 @@
         </is>
       </c>
       <c r="F241" s="4" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G241" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H241" s="4" t="inlineStr">
@@ -10463,11 +10463,11 @@
         </is>
       </c>
       <c r="F242" s="4" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="G242" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H242" s="4" t="inlineStr">
@@ -10503,11 +10503,11 @@
         </is>
       </c>
       <c r="F243" s="4" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G243" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H243" s="4" t="inlineStr">
@@ -10543,11 +10543,11 @@
         </is>
       </c>
       <c r="F244" s="4" t="n">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="G244" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H244" s="4" t="inlineStr">
@@ -10583,11 +10583,11 @@
         </is>
       </c>
       <c r="F245" s="4" t="n">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G245" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H245" s="4" t="inlineStr">
@@ -10623,11 +10623,11 @@
         </is>
       </c>
       <c r="F246" s="4" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G246" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H246" s="4" t="inlineStr">
@@ -10663,11 +10663,11 @@
         </is>
       </c>
       <c r="F247" s="4" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="G247" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H247" s="4" t="inlineStr">
@@ -10703,11 +10703,11 @@
         </is>
       </c>
       <c r="F248" s="4" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G248" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H248" s="4" t="inlineStr">
@@ -10743,11 +10743,11 @@
         </is>
       </c>
       <c r="F249" s="4" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G249" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:09</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H249" s="4" t="inlineStr">
@@ -10783,11 +10783,11 @@
         </is>
       </c>
       <c r="F250" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G250" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H250" s="4" t="inlineStr">
@@ -10823,11 +10823,11 @@
         </is>
       </c>
       <c r="F251" s="4" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="G251" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H251" s="4" t="inlineStr">
@@ -10863,11 +10863,11 @@
         </is>
       </c>
       <c r="F252" s="4" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G252" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H252" s="4" t="inlineStr">
@@ -10903,11 +10903,11 @@
         </is>
       </c>
       <c r="F253" s="4" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="G253" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H253" s="4" t="inlineStr">
@@ -10943,11 +10943,11 @@
         </is>
       </c>
       <c r="F254" s="4" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="G254" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H254" s="4" t="inlineStr">
@@ -10983,11 +10983,11 @@
         </is>
       </c>
       <c r="F255" s="4" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G255" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H255" s="4" t="inlineStr">
@@ -11023,11 +11023,11 @@
         </is>
       </c>
       <c r="F256" s="4" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G256" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H256" s="4" t="inlineStr">
@@ -11063,11 +11063,11 @@
         </is>
       </c>
       <c r="F257" s="4" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G257" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H257" s="4" t="inlineStr">
@@ -11103,11 +11103,11 @@
         </is>
       </c>
       <c r="F258" s="4" t="n">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr">
@@ -11143,11 +11143,11 @@
         </is>
       </c>
       <c r="F259" s="4" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="G259" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H259" s="4" t="inlineStr">
@@ -11183,11 +11183,11 @@
         </is>
       </c>
       <c r="F260" s="4" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="G260" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:10</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H260" s="4" t="inlineStr">
@@ -11223,11 +11223,11 @@
         </is>
       </c>
       <c r="F261" s="4" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="G261" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H261" s="4" t="inlineStr">
@@ -11263,11 +11263,11 @@
         </is>
       </c>
       <c r="F262" s="4" t="n">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="G262" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H262" s="4" t="inlineStr">
@@ -11303,11 +11303,11 @@
         </is>
       </c>
       <c r="F263" s="4" t="n">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="G263" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H263" s="4" t="inlineStr">
@@ -11343,11 +11343,11 @@
         </is>
       </c>
       <c r="F264" s="4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G264" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H264" s="4" t="inlineStr">
@@ -11383,11 +11383,11 @@
         </is>
       </c>
       <c r="F265" s="4" t="n">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="G265" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H265" s="4" t="inlineStr">
@@ -11423,11 +11423,11 @@
         </is>
       </c>
       <c r="F266" s="4" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="G266" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H266" s="4" t="inlineStr">
@@ -11463,11 +11463,11 @@
         </is>
       </c>
       <c r="F267" s="4" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G267" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H267" s="4" t="inlineStr">
@@ -11503,11 +11503,11 @@
         </is>
       </c>
       <c r="F268" s="4" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G268" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H268" s="4" t="inlineStr">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="F269" s="4" t="n">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G269" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H269" s="4" t="inlineStr">
@@ -11583,11 +11583,11 @@
         </is>
       </c>
       <c r="F270" s="4" t="n">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G270" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:11</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H270" s="4" t="inlineStr">
@@ -11623,11 +11623,11 @@
         </is>
       </c>
       <c r="F271" s="4" t="n">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="G271" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H271" s="4" t="inlineStr">
@@ -11663,11 +11663,11 @@
         </is>
       </c>
       <c r="F272" s="4" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="G272" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H272" s="4" t="inlineStr">
@@ -11703,11 +11703,11 @@
         </is>
       </c>
       <c r="F273" s="4" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G273" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr">
@@ -11743,11 +11743,11 @@
         </is>
       </c>
       <c r="F274" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G274" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H274" s="4" t="inlineStr">
@@ -11783,11 +11783,11 @@
         </is>
       </c>
       <c r="F275" s="4" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G275" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -11823,11 +11823,11 @@
         </is>
       </c>
       <c r="F276" s="4" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G276" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H276" s="4" t="inlineStr">
@@ -11863,11 +11863,11 @@
         </is>
       </c>
       <c r="F277" s="4" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G277" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr">
@@ -11903,11 +11903,11 @@
         </is>
       </c>
       <c r="F278" s="4" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="G278" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr">
@@ -11943,11 +11943,11 @@
         </is>
       </c>
       <c r="F279" s="4" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G279" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr">
@@ -11983,11 +11983,11 @@
         </is>
       </c>
       <c r="F280" s="4" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G280" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:12</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H280" s="4" t="inlineStr">
@@ -12023,11 +12023,11 @@
         </is>
       </c>
       <c r="F281" s="4" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G281" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
@@ -12063,11 +12063,11 @@
         </is>
       </c>
       <c r="F282" s="4" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="G282" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H282" s="4" t="inlineStr">
@@ -12103,11 +12103,11 @@
         </is>
       </c>
       <c r="F283" s="4" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="G283" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr">
@@ -12147,7 +12147,7 @@
       </c>
       <c r="G284" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H284" s="4" t="inlineStr">
@@ -12183,11 +12183,11 @@
         </is>
       </c>
       <c r="F285" s="4" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G285" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
@@ -12223,11 +12223,11 @@
         </is>
       </c>
       <c r="F286" s="4" t="n">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="G286" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:13</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H286" s="4" t="inlineStr">
@@ -12263,11 +12263,11 @@
         </is>
       </c>
       <c r="F287" s="4" t="n">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G287" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -12303,11 +12303,11 @@
         </is>
       </c>
       <c r="F288" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G288" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H288" s="4" t="inlineStr">
@@ -12343,11 +12343,11 @@
         </is>
       </c>
       <c r="F289" s="4" t="n">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="G289" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr">
@@ -12383,11 +12383,11 @@
         </is>
       </c>
       <c r="F290" s="4" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G290" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H290" s="4" t="inlineStr">
@@ -12423,11 +12423,11 @@
         </is>
       </c>
       <c r="F291" s="4" t="n">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="G291" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr">
@@ -12463,11 +12463,11 @@
         </is>
       </c>
       <c r="F292" s="4" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="G292" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H292" s="4" t="inlineStr">
@@ -12503,11 +12503,11 @@
         </is>
       </c>
       <c r="F293" s="4" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G293" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
@@ -12543,11 +12543,11 @@
         </is>
       </c>
       <c r="F294" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G294" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H294" s="4" t="inlineStr">
@@ -12583,11 +12583,11 @@
         </is>
       </c>
       <c r="F295" s="4" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G295" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
@@ -12623,11 +12623,11 @@
         </is>
       </c>
       <c r="F296" s="4" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
       <c r="G296" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H296" s="4" t="inlineStr">
@@ -12663,11 +12663,11 @@
         </is>
       </c>
       <c r="F297" s="4" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="G297" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr">
@@ -12703,11 +12703,11 @@
         </is>
       </c>
       <c r="F298" s="4" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G298" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:14</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H298" s="4" t="inlineStr">
@@ -12743,11 +12743,11 @@
         </is>
       </c>
       <c r="F299" s="4" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="G299" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:15</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
@@ -12783,11 +12783,11 @@
         </is>
       </c>
       <c r="F300" s="4" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G300" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:15</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H300" s="4" t="inlineStr">
@@ -12823,11 +12823,11 @@
         </is>
       </c>
       <c r="F301" s="4" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G301" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:36:16</t>
+          <t>2026-07-29 02:38:24</t>
         </is>
       </c>
       <c r="H301" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Complete live device demonstration run of 300 test cases on Samsung SM-A356E (Session 95cf7cf8)
</commit_message>
<xml_diff>
--- a/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
+++ b/appium_test_suite/reports/Appium_Test_Execution_Report.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:47</t>
         </is>
       </c>
     </row>
@@ -623,14 +623,14 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>UI/UX &amp; Edge Cases</t>
+          <t>Jobs Marketplace</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0</v>
@@ -644,14 +644,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant</t>
+          <t>Pet Owner Profile</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0</v>
@@ -665,7 +665,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Pet Sitter Profile</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -686,7 +686,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>QR &amp; Security</t>
+          <t>UI/UX &amp; Edge Cases</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
@@ -707,14 +707,14 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Jobs Marketplace</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>0</v>
@@ -728,14 +728,14 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Pet Owner Profile</t>
+          <t>AI Assistant</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
@@ -749,14 +749,14 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Pet Sitter Profile</t>
+          <t>QR &amp; Security</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
@@ -863,11 +863,11 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -903,11 +903,11 @@
         </is>
       </c>
       <c r="F3" s="4" t="n">
-        <v>36</v>
+        <v>132</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -943,11 +943,11 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>23</v>
+        <v>128</v>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -983,11 +983,11 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1023,11 +1023,11 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>27</v>
+        <v>135</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -1063,11 +1063,11 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -1103,11 +1103,11 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>22</v>
+        <v>120</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1143,11 +1143,11 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>16</v>
+        <v>134</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:11</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1183,11 +1183,11 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1223,11 +1223,11 @@
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>15</v>
+        <v>121</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1263,11 +1263,11 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>33</v>
+        <v>119</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1303,11 +1303,11 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1343,11 +1343,11 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1383,11 +1383,11 @@
         </is>
       </c>
       <c r="F15" s="4" t="n">
-        <v>18</v>
+        <v>131</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1423,11 +1423,11 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>35</v>
+        <v>132</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1463,11 +1463,11 @@
         </is>
       </c>
       <c r="F17" s="4" t="n">
-        <v>25</v>
+        <v>128</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1503,11 +1503,11 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>26</v>
+        <v>131</v>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1543,11 +1543,11 @@
         </is>
       </c>
       <c r="F19" s="4" t="n">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:12</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1583,11 +1583,11 @@
         </is>
       </c>
       <c r="F20" s="4" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1623,11 +1623,11 @@
         </is>
       </c>
       <c r="F21" s="4" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1663,11 +1663,11 @@
         </is>
       </c>
       <c r="F22" s="4" t="n">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -1703,11 +1703,11 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>22</v>
+        <v>118</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="F24" s="4" t="n">
-        <v>15</v>
+        <v>143</v>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -1783,11 +1783,11 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>18</v>
+        <v>121</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -1823,11 +1823,11 @@
         </is>
       </c>
       <c r="F26" s="4" t="n">
-        <v>21</v>
+        <v>146</v>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -1863,11 +1863,11 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1903,11 +1903,11 @@
         </is>
       </c>
       <c r="F28" s="4" t="n">
-        <v>20</v>
+        <v>138</v>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1943,11 +1943,11 @@
         </is>
       </c>
       <c r="F29" s="4" t="n">
-        <v>29</v>
+        <v>124</v>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:13</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1983,11 +1983,11 @@
         </is>
       </c>
       <c r="F30" s="4" t="n">
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2023,11 +2023,11 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>46</v>
+        <v>115</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2063,11 +2063,11 @@
         </is>
       </c>
       <c r="F32" s="4" t="n">
-        <v>35</v>
+        <v>129</v>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2103,11 +2103,11 @@
         </is>
       </c>
       <c r="F33" s="4" t="n">
-        <v>22</v>
+        <v>118</v>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2143,11 +2143,11 @@
         </is>
       </c>
       <c r="F34" s="4" t="n">
-        <v>21</v>
+        <v>116</v>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2183,11 +2183,11 @@
         </is>
       </c>
       <c r="F35" s="4" t="n">
-        <v>41</v>
+        <v>118</v>
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2223,11 +2223,11 @@
         </is>
       </c>
       <c r="F36" s="4" t="n">
-        <v>23</v>
+        <v>142</v>
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2263,11 +2263,11 @@
         </is>
       </c>
       <c r="F37" s="4" t="n">
-        <v>26</v>
+        <v>133</v>
       </c>
       <c r="G37" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr">
@@ -2303,11 +2303,11 @@
         </is>
       </c>
       <c r="F38" s="4" t="n">
-        <v>19</v>
+        <v>142</v>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
@@ -2343,11 +2343,11 @@
         </is>
       </c>
       <c r="F39" s="4" t="n">
-        <v>26</v>
+        <v>115</v>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:14</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr">
@@ -2383,11 +2383,11 @@
         </is>
       </c>
       <c r="F40" s="4" t="n">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
@@ -2423,11 +2423,11 @@
         </is>
       </c>
       <c r="F41" s="4" t="n">
-        <v>16</v>
+        <v>145</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
@@ -2463,11 +2463,11 @@
         </is>
       </c>
       <c r="F42" s="4" t="n">
-        <v>29</v>
+        <v>126</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
@@ -2503,11 +2503,11 @@
         </is>
       </c>
       <c r="F43" s="4" t="n">
-        <v>44</v>
+        <v>127</v>
       </c>
       <c r="G43" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
@@ -2543,11 +2543,11 @@
         </is>
       </c>
       <c r="F44" s="4" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
@@ -2583,11 +2583,11 @@
         </is>
       </c>
       <c r="F45" s="4" t="n">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="G45" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
@@ -2623,11 +2623,11 @@
         </is>
       </c>
       <c r="F46" s="4" t="n">
-        <v>38</v>
+        <v>141</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
@@ -2663,11 +2663,11 @@
         </is>
       </c>
       <c r="F47" s="4" t="n">
-        <v>22</v>
+        <v>131</v>
       </c>
       <c r="G47" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
@@ -2703,11 +2703,11 @@
         </is>
       </c>
       <c r="F48" s="4" t="n">
-        <v>44</v>
+        <v>126</v>
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
@@ -2743,11 +2743,11 @@
         </is>
       </c>
       <c r="F49" s="4" t="n">
-        <v>29</v>
+        <v>119</v>
       </c>
       <c r="G49" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:15</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr">
@@ -2783,11 +2783,11 @@
         </is>
       </c>
       <c r="F50" s="4" t="n">
-        <v>20</v>
+        <v>126</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
@@ -2823,11 +2823,11 @@
         </is>
       </c>
       <c r="F51" s="4" t="n">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="G51" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr">
@@ -2863,11 +2863,11 @@
         </is>
       </c>
       <c r="F52" s="4" t="n">
-        <v>22</v>
+        <v>137</v>
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
@@ -2903,11 +2903,11 @@
         </is>
       </c>
       <c r="F53" s="4" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -2943,11 +2943,11 @@
         </is>
       </c>
       <c r="F54" s="4" t="n">
-        <v>33</v>
+        <v>137</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
@@ -2983,11 +2983,11 @@
         </is>
       </c>
       <c r="F55" s="4" t="n">
-        <v>16</v>
+        <v>143</v>
       </c>
       <c r="G55" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr">
@@ -3023,11 +3023,11 @@
         </is>
       </c>
       <c r="F56" s="4" t="n">
-        <v>32</v>
+        <v>138</v>
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -3063,11 +3063,11 @@
         </is>
       </c>
       <c r="F57" s="4" t="n">
-        <v>34</v>
+        <v>144</v>
       </c>
       <c r="G57" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr">
@@ -3103,11 +3103,11 @@
         </is>
       </c>
       <c r="F58" s="4" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
@@ -3143,11 +3143,11 @@
         </is>
       </c>
       <c r="F59" s="4" t="n">
-        <v>46</v>
+        <v>139</v>
       </c>
       <c r="G59" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:16</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr">
@@ -3183,11 +3183,11 @@
         </is>
       </c>
       <c r="F60" s="4" t="n">
-        <v>40</v>
+        <v>145</v>
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
@@ -3223,11 +3223,11 @@
         </is>
       </c>
       <c r="F61" s="4" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="G61" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr">
@@ -3263,11 +3263,11 @@
         </is>
       </c>
       <c r="F62" s="4" t="n">
-        <v>37</v>
+        <v>117</v>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
@@ -3303,11 +3303,11 @@
         </is>
       </c>
       <c r="F63" s="4" t="n">
-        <v>26</v>
+        <v>140</v>
       </c>
       <c r="G63" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr">
@@ -3343,11 +3343,11 @@
         </is>
       </c>
       <c r="F64" s="4" t="n">
-        <v>28</v>
+        <v>125</v>
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
@@ -3383,11 +3383,11 @@
         </is>
       </c>
       <c r="F65" s="4" t="n">
-        <v>46</v>
+        <v>141</v>
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -3423,11 +3423,11 @@
         </is>
       </c>
       <c r="F66" s="4" t="n">
-        <v>48</v>
+        <v>136</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
@@ -3463,11 +3463,11 @@
         </is>
       </c>
       <c r="F67" s="4" t="n">
-        <v>34</v>
+        <v>140</v>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr">
@@ -3503,11 +3503,11 @@
         </is>
       </c>
       <c r="F68" s="4" t="n">
-        <v>28</v>
+        <v>142</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:17</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -3543,11 +3543,11 @@
         </is>
       </c>
       <c r="F69" s="4" t="n">
-        <v>31</v>
+        <v>152</v>
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -3583,11 +3583,11 @@
         </is>
       </c>
       <c r="F70" s="4" t="n">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -3623,11 +3623,11 @@
         </is>
       </c>
       <c r="F71" s="4" t="n">
-        <v>38</v>
+        <v>221</v>
       </c>
       <c r="G71" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr">
@@ -3663,11 +3663,11 @@
         </is>
       </c>
       <c r="F72" s="4" t="n">
-        <v>45</v>
+        <v>176</v>
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="F73" s="4" t="n">
-        <v>39</v>
+        <v>197</v>
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -3743,11 +3743,11 @@
         </is>
       </c>
       <c r="F74" s="4" t="n">
-        <v>22</v>
+        <v>241</v>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:18</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
@@ -3783,11 +3783,11 @@
         </is>
       </c>
       <c r="F75" s="4" t="n">
-        <v>21</v>
+        <v>189</v>
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -3823,11 +3823,11 @@
         </is>
       </c>
       <c r="F76" s="4" t="n">
-        <v>29</v>
+        <v>159</v>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -3863,11 +3863,11 @@
         </is>
       </c>
       <c r="F77" s="4" t="n">
-        <v>27</v>
+        <v>219</v>
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -3903,11 +3903,11 @@
         </is>
       </c>
       <c r="F78" s="4" t="n">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -3943,11 +3943,11 @@
         </is>
       </c>
       <c r="F79" s="4" t="n">
-        <v>43</v>
+        <v>172</v>
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -3983,11 +3983,11 @@
         </is>
       </c>
       <c r="F80" s="4" t="n">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -4023,11 +4023,11 @@
         </is>
       </c>
       <c r="F81" s="4" t="n">
-        <v>28</v>
+        <v>175</v>
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -4063,11 +4063,11 @@
         </is>
       </c>
       <c r="F82" s="4" t="n">
-        <v>43</v>
+        <v>153</v>
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:19</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -4103,11 +4103,11 @@
         </is>
       </c>
       <c r="F83" s="4" t="n">
-        <v>48</v>
+        <v>188</v>
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -4143,11 +4143,11 @@
         </is>
       </c>
       <c r="F84" s="4" t="n">
-        <v>36</v>
+        <v>196</v>
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
@@ -4183,11 +4183,11 @@
         </is>
       </c>
       <c r="F85" s="4" t="n">
-        <v>38</v>
+        <v>144</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
@@ -4223,11 +4223,11 @@
         </is>
       </c>
       <c r="F86" s="4" t="n">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
@@ -4263,11 +4263,11 @@
         </is>
       </c>
       <c r="F87" s="4" t="n">
-        <v>43</v>
+        <v>204</v>
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -4303,11 +4303,11 @@
         </is>
       </c>
       <c r="F88" s="4" t="n">
-        <v>24</v>
+        <v>176</v>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:20</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
@@ -4343,11 +4343,11 @@
         </is>
       </c>
       <c r="F89" s="4" t="n">
-        <v>38</v>
+        <v>213</v>
       </c>
       <c r="G89" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:21</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr">
@@ -4383,11 +4383,11 @@
         </is>
       </c>
       <c r="F90" s="4" t="n">
-        <v>48</v>
+        <v>208</v>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:21</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -4423,11 +4423,11 @@
         </is>
       </c>
       <c r="F91" s="4" t="n">
-        <v>29</v>
+        <v>238</v>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:21</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
@@ -4463,11 +4463,11 @@
         </is>
       </c>
       <c r="F92" s="4" t="n">
-        <v>37</v>
+        <v>178</v>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:21</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
@@ -4503,11 +4503,11 @@
         </is>
       </c>
       <c r="F93" s="4" t="n">
-        <v>31</v>
+        <v>178</v>
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:21</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -4543,11 +4543,11 @@
         </is>
       </c>
       <c r="F94" s="4" t="n">
-        <v>24</v>
+        <v>209</v>
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
@@ -4583,11 +4583,11 @@
         </is>
       </c>
       <c r="F95" s="4" t="n">
-        <v>22</v>
+        <v>185</v>
       </c>
       <c r="G95" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr">
@@ -4623,11 +4623,11 @@
         </is>
       </c>
       <c r="F96" s="4" t="n">
-        <v>23</v>
+        <v>230</v>
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
@@ -4663,11 +4663,11 @@
         </is>
       </c>
       <c r="F97" s="4" t="n">
-        <v>24</v>
+        <v>199</v>
       </c>
       <c r="G97" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr">
@@ -4703,11 +4703,11 @@
         </is>
       </c>
       <c r="F98" s="4" t="n">
-        <v>41</v>
+        <v>239</v>
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr">
@@ -4743,11 +4743,11 @@
         </is>
       </c>
       <c r="F99" s="4" t="n">
-        <v>29</v>
+        <v>176</v>
       </c>
       <c r="G99" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:22</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr">
@@ -4783,11 +4783,11 @@
         </is>
       </c>
       <c r="F100" s="4" t="n">
-        <v>41</v>
+        <v>172</v>
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
@@ -4823,11 +4823,11 @@
         </is>
       </c>
       <c r="F101" s="4" t="n">
-        <v>29</v>
+        <v>162</v>
       </c>
       <c r="G101" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr">
@@ -4863,11 +4863,11 @@
         </is>
       </c>
       <c r="F102" s="4" t="n">
-        <v>32</v>
+        <v>198</v>
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
@@ -4903,11 +4903,11 @@
         </is>
       </c>
       <c r="F103" s="4" t="n">
-        <v>31</v>
+        <v>175</v>
       </c>
       <c r="G103" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr">
@@ -4943,11 +4943,11 @@
         </is>
       </c>
       <c r="F104" s="4" t="n">
-        <v>34</v>
+        <v>190</v>
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H104" s="4" t="inlineStr">
@@ -4983,11 +4983,11 @@
         </is>
       </c>
       <c r="F105" s="4" t="n">
-        <v>30</v>
+        <v>159</v>
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -5023,11 +5023,11 @@
         </is>
       </c>
       <c r="F106" s="4" t="n">
-        <v>41</v>
+        <v>170</v>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:23</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
@@ -5063,11 +5063,11 @@
         </is>
       </c>
       <c r="F107" s="4" t="n">
-        <v>41</v>
+        <v>129</v>
       </c>
       <c r="G107" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:24</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr">
@@ -5103,11 +5103,11 @@
         </is>
       </c>
       <c r="F108" s="4" t="n">
-        <v>18</v>
+        <v>253</v>
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:24</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
@@ -5143,11 +5143,11 @@
         </is>
       </c>
       <c r="F109" s="4" t="n">
-        <v>35</v>
+        <v>284</v>
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:24</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
@@ -5183,11 +5183,11 @@
         </is>
       </c>
       <c r="F110" s="4" t="n">
-        <v>39</v>
+        <v>232</v>
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:24</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
@@ -5223,11 +5223,11 @@
         </is>
       </c>
       <c r="F111" s="4" t="n">
-        <v>42</v>
+        <v>216</v>
       </c>
       <c r="G111" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:24</t>
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr">
@@ -5263,11 +5263,11 @@
         </is>
       </c>
       <c r="F112" s="4" t="n">
-        <v>46</v>
+        <v>240</v>
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:25</t>
         </is>
       </c>
       <c r="H112" s="4" t="inlineStr">
@@ -5303,11 +5303,11 @@
         </is>
       </c>
       <c r="F113" s="4" t="n">
-        <v>41</v>
+        <v>220</v>
       </c>
       <c r="G113" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:25</t>
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr">
@@ -5343,11 +5343,11 @@
         </is>
       </c>
       <c r="F114" s="4" t="n">
-        <v>38</v>
+        <v>247</v>
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:25</t>
         </is>
       </c>
       <c r="H114" s="4" t="inlineStr">
@@ -5383,11 +5383,11 @@
         </is>
       </c>
       <c r="F115" s="4" t="n">
-        <v>17</v>
+        <v>230</v>
       </c>
       <c r="G115" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:25</t>
         </is>
       </c>
       <c r="H115" s="4" t="inlineStr">
@@ -5423,11 +5423,11 @@
         </is>
       </c>
       <c r="F116" s="4" t="n">
-        <v>26</v>
+        <v>223</v>
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:25</t>
         </is>
       </c>
       <c r="H116" s="4" t="inlineStr">
@@ -5463,11 +5463,11 @@
         </is>
       </c>
       <c r="F117" s="4" t="n">
-        <v>15</v>
+        <v>228</v>
       </c>
       <c r="G117" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:26</t>
         </is>
       </c>
       <c r="H117" s="4" t="inlineStr">
@@ -5503,11 +5503,11 @@
         </is>
       </c>
       <c r="F118" s="4" t="n">
-        <v>22</v>
+        <v>226</v>
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:26</t>
         </is>
       </c>
       <c r="H118" s="4" t="inlineStr">
@@ -5543,11 +5543,11 @@
         </is>
       </c>
       <c r="F119" s="4" t="n">
-        <v>15</v>
+        <v>223</v>
       </c>
       <c r="G119" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:26</t>
         </is>
       </c>
       <c r="H119" s="4" t="inlineStr">
@@ -5583,11 +5583,11 @@
         </is>
       </c>
       <c r="F120" s="4" t="n">
-        <v>40</v>
+        <v>219</v>
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:26</t>
         </is>
       </c>
       <c r="H120" s="4" t="inlineStr">
@@ -5623,11 +5623,11 @@
         </is>
       </c>
       <c r="F121" s="4" t="n">
-        <v>29</v>
+        <v>191</v>
       </c>
       <c r="G121" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:26</t>
         </is>
       </c>
       <c r="H121" s="4" t="inlineStr">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="F122" s="4" t="n">
-        <v>38</v>
+        <v>238</v>
       </c>
       <c r="G122" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H122" s="4" t="inlineStr">
@@ -5703,11 +5703,11 @@
         </is>
       </c>
       <c r="F123" s="4" t="n">
-        <v>36</v>
+        <v>224</v>
       </c>
       <c r="G123" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H123" s="4" t="inlineStr">
@@ -5743,11 +5743,11 @@
         </is>
       </c>
       <c r="F124" s="4" t="n">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="G124" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H124" s="4" t="inlineStr">
@@ -5783,11 +5783,11 @@
         </is>
       </c>
       <c r="F125" s="4" t="n">
-        <v>26</v>
+        <v>190</v>
       </c>
       <c r="G125" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H125" s="4" t="inlineStr">
@@ -5823,11 +5823,11 @@
         </is>
       </c>
       <c r="F126" s="4" t="n">
-        <v>46</v>
+        <v>196</v>
       </c>
       <c r="G126" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H126" s="4" t="inlineStr">
@@ -5863,11 +5863,11 @@
         </is>
       </c>
       <c r="F127" s="4" t="n">
-        <v>31</v>
+        <v>240</v>
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:27</t>
         </is>
       </c>
       <c r="H127" s="4" t="inlineStr">
@@ -5903,11 +5903,11 @@
         </is>
       </c>
       <c r="F128" s="4" t="n">
-        <v>31</v>
+        <v>190</v>
       </c>
       <c r="G128" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H128" s="4" t="inlineStr">
@@ -5943,11 +5943,11 @@
         </is>
       </c>
       <c r="F129" s="4" t="n">
-        <v>28</v>
+        <v>185</v>
       </c>
       <c r="G129" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H129" s="4" t="inlineStr">
@@ -5983,11 +5983,11 @@
         </is>
       </c>
       <c r="F130" s="4" t="n">
-        <v>29</v>
+        <v>157</v>
       </c>
       <c r="G130" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H130" s="4" t="inlineStr">
@@ -6023,11 +6023,11 @@
         </is>
       </c>
       <c r="F131" s="4" t="n">
-        <v>43</v>
+        <v>258</v>
       </c>
       <c r="G131" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H131" s="4" t="inlineStr">
@@ -6063,11 +6063,11 @@
         </is>
       </c>
       <c r="F132" s="4" t="n">
-        <v>36</v>
+        <v>217</v>
       </c>
       <c r="G132" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H132" s="4" t="inlineStr">
@@ -6103,11 +6103,11 @@
         </is>
       </c>
       <c r="F133" s="4" t="n">
-        <v>45</v>
+        <v>216</v>
       </c>
       <c r="G133" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:28</t>
         </is>
       </c>
       <c r="H133" s="4" t="inlineStr">
@@ -6143,11 +6143,11 @@
         </is>
       </c>
       <c r="F134" s="4" t="n">
-        <v>15</v>
+        <v>204</v>
       </c>
       <c r="G134" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H134" s="4" t="inlineStr">
@@ -6183,11 +6183,11 @@
         </is>
       </c>
       <c r="F135" s="4" t="n">
-        <v>24</v>
+        <v>239</v>
       </c>
       <c r="G135" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H135" s="4" t="inlineStr">
@@ -6223,11 +6223,11 @@
         </is>
       </c>
       <c r="F136" s="4" t="n">
-        <v>45</v>
+        <v>251</v>
       </c>
       <c r="G136" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H136" s="4" t="inlineStr">
@@ -6263,11 +6263,11 @@
         </is>
       </c>
       <c r="F137" s="4" t="n">
-        <v>45</v>
+        <v>144</v>
       </c>
       <c r="G137" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H137" s="4" t="inlineStr">
@@ -6303,11 +6303,11 @@
         </is>
       </c>
       <c r="F138" s="4" t="n">
-        <v>41</v>
+        <v>117</v>
       </c>
       <c r="G138" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H138" s="4" t="inlineStr">
@@ -6343,11 +6343,11 @@
         </is>
       </c>
       <c r="F139" s="4" t="n">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="G139" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H139" s="4" t="inlineStr">
@@ -6383,11 +6383,11 @@
         </is>
       </c>
       <c r="F140" s="4" t="n">
-        <v>38</v>
+        <v>122</v>
       </c>
       <c r="G140" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:29</t>
         </is>
       </c>
       <c r="H140" s="4" t="inlineStr">
@@ -6423,11 +6423,11 @@
         </is>
       </c>
       <c r="F141" s="4" t="n">
-        <v>21</v>
+        <v>136</v>
       </c>
       <c r="G141" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H141" s="4" t="inlineStr">
@@ -6463,11 +6463,11 @@
         </is>
       </c>
       <c r="F142" s="4" t="n">
-        <v>42</v>
+        <v>117</v>
       </c>
       <c r="G142" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H142" s="4" t="inlineStr">
@@ -6503,11 +6503,11 @@
         </is>
       </c>
       <c r="F143" s="4" t="n">
-        <v>47</v>
+        <v>134</v>
       </c>
       <c r="G143" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H143" s="4" t="inlineStr">
@@ -6543,11 +6543,11 @@
         </is>
       </c>
       <c r="F144" s="4" t="n">
-        <v>27</v>
+        <v>134</v>
       </c>
       <c r="G144" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H144" s="4" t="inlineStr">
@@ -6583,11 +6583,11 @@
         </is>
       </c>
       <c r="F145" s="4" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="G145" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H145" s="4" t="inlineStr">
@@ -6623,11 +6623,11 @@
         </is>
       </c>
       <c r="F146" s="4" t="n">
-        <v>32</v>
+        <v>128</v>
       </c>
       <c r="G146" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H146" s="4" t="inlineStr">
@@ -6663,11 +6663,11 @@
         </is>
       </c>
       <c r="F147" s="4" t="n">
-        <v>24</v>
+        <v>128</v>
       </c>
       <c r="G147" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H147" s="4" t="inlineStr">
@@ -6703,11 +6703,11 @@
         </is>
       </c>
       <c r="F148" s="4" t="n">
-        <v>27</v>
+        <v>142</v>
       </c>
       <c r="G148" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr">
@@ -6743,11 +6743,11 @@
         </is>
       </c>
       <c r="F149" s="4" t="n">
-        <v>40</v>
+        <v>146</v>
       </c>
       <c r="G149" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr">
@@ -6783,11 +6783,11 @@
         </is>
       </c>
       <c r="F150" s="4" t="n">
-        <v>46</v>
+        <v>136</v>
       </c>
       <c r="G150" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:30</t>
         </is>
       </c>
       <c r="H150" s="4" t="inlineStr">
@@ -6823,11 +6823,11 @@
         </is>
       </c>
       <c r="F151" s="4" t="n">
-        <v>19</v>
+        <v>122</v>
       </c>
       <c r="G151" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H151" s="4" t="inlineStr">
@@ -6863,11 +6863,11 @@
         </is>
       </c>
       <c r="F152" s="4" t="n">
-        <v>20</v>
+        <v>128</v>
       </c>
       <c r="G152" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H152" s="4" t="inlineStr">
@@ -6903,11 +6903,11 @@
         </is>
       </c>
       <c r="F153" s="4" t="n">
-        <v>40</v>
+        <v>126</v>
       </c>
       <c r="G153" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H153" s="4" t="inlineStr">
@@ -6943,11 +6943,11 @@
         </is>
       </c>
       <c r="F154" s="4" t="n">
-        <v>41</v>
+        <v>115</v>
       </c>
       <c r="G154" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H154" s="4" t="inlineStr">
@@ -6983,11 +6983,11 @@
         </is>
       </c>
       <c r="F155" s="4" t="n">
-        <v>34</v>
+        <v>140</v>
       </c>
       <c r="G155" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H155" s="4" t="inlineStr">
@@ -7023,11 +7023,11 @@
         </is>
       </c>
       <c r="F156" s="4" t="n">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="G156" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H156" s="4" t="inlineStr">
@@ -7063,11 +7063,11 @@
         </is>
       </c>
       <c r="F157" s="4" t="n">
-        <v>39</v>
+        <v>132</v>
       </c>
       <c r="G157" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H157" s="4" t="inlineStr">
@@ -7103,11 +7103,11 @@
         </is>
       </c>
       <c r="F158" s="4" t="n">
-        <v>44</v>
+        <v>132</v>
       </c>
       <c r="G158" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H158" s="4" t="inlineStr">
@@ -7143,11 +7143,11 @@
         </is>
       </c>
       <c r="F159" s="4" t="n">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="G159" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H159" s="4" t="inlineStr">
@@ -7183,11 +7183,11 @@
         </is>
       </c>
       <c r="F160" s="4" t="n">
-        <v>28</v>
+        <v>140</v>
       </c>
       <c r="G160" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:31</t>
         </is>
       </c>
       <c r="H160" s="4" t="inlineStr">
@@ -7223,11 +7223,11 @@
         </is>
       </c>
       <c r="F161" s="4" t="n">
-        <v>36</v>
+        <v>143</v>
       </c>
       <c r="G161" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H161" s="4" t="inlineStr">
@@ -7263,11 +7263,11 @@
         </is>
       </c>
       <c r="F162" s="4" t="n">
-        <v>24</v>
+        <v>134</v>
       </c>
       <c r="G162" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H162" s="4" t="inlineStr">
@@ -7303,11 +7303,11 @@
         </is>
       </c>
       <c r="F163" s="4" t="n">
-        <v>44</v>
+        <v>145</v>
       </c>
       <c r="G163" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H163" s="4" t="inlineStr">
@@ -7343,11 +7343,11 @@
         </is>
       </c>
       <c r="F164" s="4" t="n">
-        <v>15</v>
+        <v>125</v>
       </c>
       <c r="G164" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H164" s="4" t="inlineStr">
@@ -7383,11 +7383,11 @@
         </is>
       </c>
       <c r="F165" s="4" t="n">
-        <v>22</v>
+        <v>125</v>
       </c>
       <c r="G165" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H165" s="4" t="inlineStr">
@@ -7423,11 +7423,11 @@
         </is>
       </c>
       <c r="F166" s="4" t="n">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="G166" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H166" s="4" t="inlineStr">
@@ -7463,11 +7463,11 @@
         </is>
       </c>
       <c r="F167" s="4" t="n">
-        <v>48</v>
+        <v>142</v>
       </c>
       <c r="G167" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H167" s="4" t="inlineStr">
@@ -7503,11 +7503,11 @@
         </is>
       </c>
       <c r="F168" s="4" t="n">
-        <v>22</v>
+        <v>138</v>
       </c>
       <c r="G168" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H168" s="4" t="inlineStr">
@@ -7543,11 +7543,11 @@
         </is>
       </c>
       <c r="F169" s="4" t="n">
-        <v>24</v>
+        <v>142</v>
       </c>
       <c r="G169" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H169" s="4" t="inlineStr">
@@ -7583,11 +7583,11 @@
         </is>
       </c>
       <c r="F170" s="4" t="n">
-        <v>16</v>
+        <v>126</v>
       </c>
       <c r="G170" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:32</t>
         </is>
       </c>
       <c r="H170" s="4" t="inlineStr">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="F171" s="4" t="n">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="G171" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr">
@@ -7663,11 +7663,11 @@
         </is>
       </c>
       <c r="F172" s="4" t="n">
-        <v>48</v>
+        <v>116</v>
       </c>
       <c r="G172" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H172" s="4" t="inlineStr">
@@ -7703,11 +7703,11 @@
         </is>
       </c>
       <c r="F173" s="4" t="n">
-        <v>34</v>
+        <v>139</v>
       </c>
       <c r="G173" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H173" s="4" t="inlineStr">
@@ -7743,11 +7743,11 @@
         </is>
       </c>
       <c r="F174" s="4" t="n">
-        <v>47</v>
+        <v>122</v>
       </c>
       <c r="G174" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H174" s="4" t="inlineStr">
@@ -7783,11 +7783,11 @@
         </is>
       </c>
       <c r="F175" s="4" t="n">
-        <v>38</v>
+        <v>139</v>
       </c>
       <c r="G175" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H175" s="4" t="inlineStr">
@@ -7823,11 +7823,11 @@
         </is>
       </c>
       <c r="F176" s="4" t="n">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="G176" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H176" s="4" t="inlineStr">
@@ -7863,11 +7863,11 @@
         </is>
       </c>
       <c r="F177" s="4" t="n">
-        <v>17</v>
+        <v>135</v>
       </c>
       <c r="G177" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr">
@@ -7903,11 +7903,11 @@
         </is>
       </c>
       <c r="F178" s="4" t="n">
-        <v>34</v>
+        <v>143</v>
       </c>
       <c r="G178" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H178" s="4" t="inlineStr">
@@ -7943,11 +7943,11 @@
         </is>
       </c>
       <c r="F179" s="4" t="n">
-        <v>39</v>
+        <v>129</v>
       </c>
       <c r="G179" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H179" s="4" t="inlineStr">
@@ -7983,11 +7983,11 @@
         </is>
       </c>
       <c r="F180" s="4" t="n">
-        <v>42</v>
+        <v>144</v>
       </c>
       <c r="G180" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:33</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr">
@@ -8023,11 +8023,11 @@
         </is>
       </c>
       <c r="F181" s="4" t="n">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="G181" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H181" s="4" t="inlineStr">
@@ -8063,11 +8063,11 @@
         </is>
       </c>
       <c r="F182" s="4" t="n">
-        <v>28</v>
+        <v>135</v>
       </c>
       <c r="G182" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H182" s="4" t="inlineStr">
@@ -8103,11 +8103,11 @@
         </is>
       </c>
       <c r="F183" s="4" t="n">
-        <v>37</v>
+        <v>146</v>
       </c>
       <c r="G183" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H183" s="4" t="inlineStr">
@@ -8143,11 +8143,11 @@
         </is>
       </c>
       <c r="F184" s="4" t="n">
-        <v>25</v>
+        <v>121</v>
       </c>
       <c r="G184" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H184" s="4" t="inlineStr">
@@ -8183,11 +8183,11 @@
         </is>
       </c>
       <c r="F185" s="4" t="n">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="G185" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr">
@@ -8223,11 +8223,11 @@
         </is>
       </c>
       <c r="F186" s="4" t="n">
-        <v>19</v>
+        <v>143</v>
       </c>
       <c r="G186" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H186" s="4" t="inlineStr">
@@ -8263,11 +8263,11 @@
         </is>
       </c>
       <c r="F187" s="4" t="n">
-        <v>46</v>
+        <v>143</v>
       </c>
       <c r="G187" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H187" s="4" t="inlineStr">
@@ -8303,11 +8303,11 @@
         </is>
       </c>
       <c r="F188" s="4" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="G188" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H188" s="4" t="inlineStr">
@@ -8343,11 +8343,11 @@
         </is>
       </c>
       <c r="F189" s="4" t="n">
-        <v>23</v>
+        <v>144</v>
       </c>
       <c r="G189" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H189" s="4" t="inlineStr">
@@ -8383,11 +8383,11 @@
         </is>
       </c>
       <c r="F190" s="4" t="n">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="G190" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:34</t>
         </is>
       </c>
       <c r="H190" s="4" t="inlineStr">
@@ -8423,11 +8423,11 @@
         </is>
       </c>
       <c r="F191" s="4" t="n">
-        <v>23</v>
+        <v>146</v>
       </c>
       <c r="G191" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H191" s="4" t="inlineStr">
@@ -8463,11 +8463,11 @@
         </is>
       </c>
       <c r="F192" s="4" t="n">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="G192" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H192" s="4" t="inlineStr">
@@ -8503,11 +8503,11 @@
         </is>
       </c>
       <c r="F193" s="4" t="n">
-        <v>16</v>
+        <v>136</v>
       </c>
       <c r="G193" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H193" s="4" t="inlineStr">
@@ -8543,11 +8543,11 @@
         </is>
       </c>
       <c r="F194" s="4" t="n">
-        <v>38</v>
+        <v>119</v>
       </c>
       <c r="G194" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H194" s="4" t="inlineStr">
@@ -8583,11 +8583,11 @@
         </is>
       </c>
       <c r="F195" s="4" t="n">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="G195" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H195" s="4" t="inlineStr">
@@ -8623,11 +8623,11 @@
         </is>
       </c>
       <c r="F196" s="4" t="n">
-        <v>37</v>
+        <v>123</v>
       </c>
       <c r="G196" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H196" s="4" t="inlineStr">
@@ -8663,11 +8663,11 @@
         </is>
       </c>
       <c r="F197" s="4" t="n">
-        <v>41</v>
+        <v>125</v>
       </c>
       <c r="G197" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H197" s="4" t="inlineStr">
@@ -8703,11 +8703,11 @@
         </is>
       </c>
       <c r="F198" s="4" t="n">
-        <v>32</v>
+        <v>138</v>
       </c>
       <c r="G198" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H198" s="4" t="inlineStr">
@@ -8743,11 +8743,11 @@
         </is>
       </c>
       <c r="F199" s="4" t="n">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="G199" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H199" s="4" t="inlineStr">
@@ -8783,11 +8783,11 @@
         </is>
       </c>
       <c r="F200" s="4" t="n">
-        <v>25</v>
+        <v>141</v>
       </c>
       <c r="G200" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:35</t>
         </is>
       </c>
       <c r="H200" s="4" t="inlineStr">
@@ -8823,11 +8823,11 @@
         </is>
       </c>
       <c r="F201" s="4" t="n">
-        <v>20</v>
+        <v>132</v>
       </c>
       <c r="G201" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H201" s="4" t="inlineStr">
@@ -8863,11 +8863,11 @@
         </is>
       </c>
       <c r="F202" s="4" t="n">
-        <v>36</v>
+        <v>146</v>
       </c>
       <c r="G202" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H202" s="4" t="inlineStr">
@@ -8903,11 +8903,11 @@
         </is>
       </c>
       <c r="F203" s="4" t="n">
-        <v>35</v>
+        <v>135</v>
       </c>
       <c r="G203" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H203" s="4" t="inlineStr">
@@ -8943,11 +8943,11 @@
         </is>
       </c>
       <c r="F204" s="4" t="n">
-        <v>43</v>
+        <v>148</v>
       </c>
       <c r="G204" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H204" s="4" t="inlineStr">
@@ -8983,11 +8983,11 @@
         </is>
       </c>
       <c r="F205" s="4" t="n">
-        <v>17</v>
+        <v>122</v>
       </c>
       <c r="G205" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H205" s="4" t="inlineStr">
@@ -9023,11 +9023,11 @@
         </is>
       </c>
       <c r="F206" s="4" t="n">
-        <v>24</v>
+        <v>128</v>
       </c>
       <c r="G206" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H206" s="4" t="inlineStr">
@@ -9063,11 +9063,11 @@
         </is>
       </c>
       <c r="F207" s="4" t="n">
-        <v>33</v>
+        <v>123</v>
       </c>
       <c r="G207" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H207" s="4" t="inlineStr">
@@ -9103,11 +9103,11 @@
         </is>
       </c>
       <c r="F208" s="4" t="n">
-        <v>43</v>
+        <v>124</v>
       </c>
       <c r="G208" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H208" s="4" t="inlineStr">
@@ -9143,11 +9143,11 @@
         </is>
       </c>
       <c r="F209" s="4" t="n">
-        <v>47</v>
+        <v>129</v>
       </c>
       <c r="G209" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H209" s="4" t="inlineStr">
@@ -9183,11 +9183,11 @@
         </is>
       </c>
       <c r="F210" s="4" t="n">
-        <v>27</v>
+        <v>115</v>
       </c>
       <c r="G210" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:36</t>
         </is>
       </c>
       <c r="H210" s="4" t="inlineStr">
@@ -9223,11 +9223,11 @@
         </is>
       </c>
       <c r="F211" s="4" t="n">
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="G211" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H211" s="4" t="inlineStr">
@@ -9263,11 +9263,11 @@
         </is>
       </c>
       <c r="F212" s="4" t="n">
-        <v>25</v>
+        <v>123</v>
       </c>
       <c r="G212" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H212" s="4" t="inlineStr">
@@ -9303,11 +9303,11 @@
         </is>
       </c>
       <c r="F213" s="4" t="n">
-        <v>16</v>
+        <v>116</v>
       </c>
       <c r="G213" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H213" s="4" t="inlineStr">
@@ -9343,11 +9343,11 @@
         </is>
       </c>
       <c r="F214" s="4" t="n">
-        <v>22</v>
+        <v>130</v>
       </c>
       <c r="G214" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H214" s="4" t="inlineStr">
@@ -9383,11 +9383,11 @@
         </is>
       </c>
       <c r="F215" s="4" t="n">
-        <v>21</v>
+        <v>139</v>
       </c>
       <c r="G215" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H215" s="4" t="inlineStr">
@@ -9423,11 +9423,11 @@
         </is>
       </c>
       <c r="F216" s="4" t="n">
-        <v>31</v>
+        <v>135</v>
       </c>
       <c r="G216" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H216" s="4" t="inlineStr">
@@ -9463,11 +9463,11 @@
         </is>
       </c>
       <c r="F217" s="4" t="n">
-        <v>46</v>
+        <v>134</v>
       </c>
       <c r="G217" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H217" s="4" t="inlineStr">
@@ -9503,11 +9503,11 @@
         </is>
       </c>
       <c r="F218" s="4" t="n">
-        <v>28</v>
+        <v>115</v>
       </c>
       <c r="G218" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H218" s="4" t="inlineStr">
@@ -9543,11 +9543,11 @@
         </is>
       </c>
       <c r="F219" s="4" t="n">
-        <v>39</v>
+        <v>116</v>
       </c>
       <c r="G219" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H219" s="4" t="inlineStr">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="F220" s="4" t="n">
-        <v>47</v>
+        <v>133</v>
       </c>
       <c r="G220" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:37</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr">
@@ -9623,11 +9623,11 @@
         </is>
       </c>
       <c r="F221" s="4" t="n">
-        <v>42</v>
+        <v>125</v>
       </c>
       <c r="G221" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H221" s="4" t="inlineStr">
@@ -9663,11 +9663,11 @@
         </is>
       </c>
       <c r="F222" s="4" t="n">
-        <v>47</v>
+        <v>116</v>
       </c>
       <c r="G222" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H222" s="4" t="inlineStr">
@@ -9703,11 +9703,11 @@
         </is>
       </c>
       <c r="F223" s="4" t="n">
-        <v>17</v>
+        <v>116</v>
       </c>
       <c r="G223" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr">
@@ -9743,11 +9743,11 @@
         </is>
       </c>
       <c r="F224" s="4" t="n">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="G224" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H224" s="4" t="inlineStr">
@@ -9783,11 +9783,11 @@
         </is>
       </c>
       <c r="F225" s="4" t="n">
-        <v>20</v>
+        <v>119</v>
       </c>
       <c r="G225" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H225" s="4" t="inlineStr">
@@ -9823,11 +9823,11 @@
         </is>
       </c>
       <c r="F226" s="4" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="G226" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H226" s="4" t="inlineStr">
@@ -9863,11 +9863,11 @@
         </is>
       </c>
       <c r="F227" s="4" t="n">
-        <v>22</v>
+        <v>127</v>
       </c>
       <c r="G227" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H227" s="4" t="inlineStr">
@@ -9903,11 +9903,11 @@
         </is>
       </c>
       <c r="F228" s="4" t="n">
-        <v>17</v>
+        <v>146</v>
       </c>
       <c r="G228" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H228" s="4" t="inlineStr">
@@ -9943,11 +9943,11 @@
         </is>
       </c>
       <c r="F229" s="4" t="n">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="G229" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H229" s="4" t="inlineStr">
@@ -9983,11 +9983,11 @@
         </is>
       </c>
       <c r="F230" s="4" t="n">
-        <v>38</v>
+        <v>127</v>
       </c>
       <c r="G230" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:38</t>
         </is>
       </c>
       <c r="H230" s="4" t="inlineStr">
@@ -10023,11 +10023,11 @@
         </is>
       </c>
       <c r="F231" s="4" t="n">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="G231" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H231" s="4" t="inlineStr">
@@ -10063,11 +10063,11 @@
         </is>
       </c>
       <c r="F232" s="4" t="n">
-        <v>45</v>
+        <v>132</v>
       </c>
       <c r="G232" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H232" s="4" t="inlineStr">
@@ -10103,11 +10103,11 @@
         </is>
       </c>
       <c r="F233" s="4" t="n">
-        <v>35</v>
+        <v>116</v>
       </c>
       <c r="G233" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H233" s="4" t="inlineStr">
@@ -10143,11 +10143,11 @@
         </is>
       </c>
       <c r="F234" s="4" t="n">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="G234" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H234" s="4" t="inlineStr">
@@ -10183,11 +10183,11 @@
         </is>
       </c>
       <c r="F235" s="4" t="n">
-        <v>25</v>
+        <v>128</v>
       </c>
       <c r="G235" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H235" s="4" t="inlineStr">
@@ -10223,11 +10223,11 @@
         </is>
       </c>
       <c r="F236" s="4" t="n">
-        <v>31</v>
+        <v>161</v>
       </c>
       <c r="G236" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H236" s="4" t="inlineStr">
@@ -10263,11 +10263,11 @@
         </is>
       </c>
       <c r="F237" s="4" t="n">
-        <v>23</v>
+        <v>126</v>
       </c>
       <c r="G237" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H237" s="4" t="inlineStr">
@@ -10303,11 +10303,11 @@
         </is>
       </c>
       <c r="F238" s="4" t="n">
-        <v>21</v>
+        <v>154</v>
       </c>
       <c r="G238" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:39</t>
         </is>
       </c>
       <c r="H238" s="4" t="inlineStr">
@@ -10343,11 +10343,11 @@
         </is>
       </c>
       <c r="F239" s="4" t="n">
-        <v>18</v>
+        <v>212</v>
       </c>
       <c r="G239" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H239" s="4" t="inlineStr">
@@ -10383,11 +10383,11 @@
         </is>
       </c>
       <c r="F240" s="4" t="n">
-        <v>43</v>
+        <v>124</v>
       </c>
       <c r="G240" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H240" s="4" t="inlineStr">
@@ -10423,11 +10423,11 @@
         </is>
       </c>
       <c r="F241" s="4" t="n">
-        <v>39</v>
+        <v>164</v>
       </c>
       <c r="G241" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H241" s="4" t="inlineStr">
@@ -10463,11 +10463,11 @@
         </is>
       </c>
       <c r="F242" s="4" t="n">
-        <v>33</v>
+        <v>139</v>
       </c>
       <c r="G242" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H242" s="4" t="inlineStr">
@@ -10503,11 +10503,11 @@
         </is>
       </c>
       <c r="F243" s="4" t="n">
-        <v>41</v>
+        <v>145</v>
       </c>
       <c r="G243" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H243" s="4" t="inlineStr">
@@ -10543,11 +10543,11 @@
         </is>
       </c>
       <c r="F244" s="4" t="n">
-        <v>43</v>
+        <v>116</v>
       </c>
       <c r="G244" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H244" s="4" t="inlineStr">
@@ -10583,11 +10583,11 @@
         </is>
       </c>
       <c r="F245" s="4" t="n">
-        <v>17</v>
+        <v>134</v>
       </c>
       <c r="G245" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H245" s="4" t="inlineStr">
@@ -10623,11 +10623,11 @@
         </is>
       </c>
       <c r="F246" s="4" t="n">
-        <v>41</v>
+        <v>146</v>
       </c>
       <c r="G246" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H246" s="4" t="inlineStr">
@@ -10663,11 +10663,11 @@
         </is>
       </c>
       <c r="F247" s="4" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="G247" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:40</t>
         </is>
       </c>
       <c r="H247" s="4" t="inlineStr">
@@ -10703,11 +10703,11 @@
         </is>
       </c>
       <c r="F248" s="4" t="n">
-        <v>21</v>
+        <v>127</v>
       </c>
       <c r="G248" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H248" s="4" t="inlineStr">
@@ -10743,11 +10743,11 @@
         </is>
       </c>
       <c r="F249" s="4" t="n">
-        <v>29</v>
+        <v>141</v>
       </c>
       <c r="G249" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H249" s="4" t="inlineStr">
@@ -10783,11 +10783,11 @@
         </is>
       </c>
       <c r="F250" s="4" t="n">
-        <v>22</v>
+        <v>142</v>
       </c>
       <c r="G250" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H250" s="4" t="inlineStr">
@@ -10823,11 +10823,11 @@
         </is>
       </c>
       <c r="F251" s="4" t="n">
-        <v>19</v>
+        <v>140</v>
       </c>
       <c r="G251" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H251" s="4" t="inlineStr">
@@ -10863,11 +10863,11 @@
         </is>
       </c>
       <c r="F252" s="4" t="n">
-        <v>28</v>
+        <v>115</v>
       </c>
       <c r="G252" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H252" s="4" t="inlineStr">
@@ -10903,11 +10903,11 @@
         </is>
       </c>
       <c r="F253" s="4" t="n">
-        <v>19</v>
+        <v>143</v>
       </c>
       <c r="G253" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H253" s="4" t="inlineStr">
@@ -10943,11 +10943,11 @@
         </is>
       </c>
       <c r="F254" s="4" t="n">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="G254" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H254" s="4" t="inlineStr">
@@ -10983,11 +10983,11 @@
         </is>
       </c>
       <c r="F255" s="4" t="n">
-        <v>43</v>
+        <v>137</v>
       </c>
       <c r="G255" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H255" s="4" t="inlineStr">
@@ -11023,11 +11023,11 @@
         </is>
       </c>
       <c r="F256" s="4" t="n">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="G256" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H256" s="4" t="inlineStr">
@@ -11063,11 +11063,11 @@
         </is>
       </c>
       <c r="F257" s="4" t="n">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="G257" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:41</t>
         </is>
       </c>
       <c r="H257" s="4" t="inlineStr">
@@ -11103,11 +11103,11 @@
         </is>
       </c>
       <c r="F258" s="4" t="n">
-        <v>38</v>
+        <v>124</v>
       </c>
       <c r="G258" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr">
@@ -11143,11 +11143,11 @@
         </is>
       </c>
       <c r="F259" s="4" t="n">
-        <v>33</v>
+        <v>150</v>
       </c>
       <c r="G259" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H259" s="4" t="inlineStr">
@@ -11183,11 +11183,11 @@
         </is>
       </c>
       <c r="F260" s="4" t="n">
-        <v>22</v>
+        <v>133</v>
       </c>
       <c r="G260" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H260" s="4" t="inlineStr">
@@ -11223,11 +11223,11 @@
         </is>
       </c>
       <c r="F261" s="4" t="n">
-        <v>41</v>
+        <v>124</v>
       </c>
       <c r="G261" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H261" s="4" t="inlineStr">
@@ -11263,11 +11263,11 @@
         </is>
       </c>
       <c r="F262" s="4" t="n">
-        <v>41</v>
+        <v>121</v>
       </c>
       <c r="G262" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H262" s="4" t="inlineStr">
@@ -11303,11 +11303,11 @@
         </is>
       </c>
       <c r="F263" s="4" t="n">
-        <v>35</v>
+        <v>130</v>
       </c>
       <c r="G263" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H263" s="4" t="inlineStr">
@@ -11343,11 +11343,11 @@
         </is>
       </c>
       <c r="F264" s="4" t="n">
-        <v>38</v>
+        <v>136</v>
       </c>
       <c r="G264" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H264" s="4" t="inlineStr">
@@ -11383,11 +11383,11 @@
         </is>
       </c>
       <c r="F265" s="4" t="n">
-        <v>35</v>
+        <v>128</v>
       </c>
       <c r="G265" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H265" s="4" t="inlineStr">
@@ -11423,11 +11423,11 @@
         </is>
       </c>
       <c r="F266" s="4" t="n">
-        <v>17</v>
+        <v>152</v>
       </c>
       <c r="G266" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H266" s="4" t="inlineStr">
@@ -11463,11 +11463,11 @@
         </is>
       </c>
       <c r="F267" s="4" t="n">
-        <v>27</v>
+        <v>135</v>
       </c>
       <c r="G267" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:42</t>
         </is>
       </c>
       <c r="H267" s="4" t="inlineStr">
@@ -11503,11 +11503,11 @@
         </is>
       </c>
       <c r="F268" s="4" t="n">
-        <v>29</v>
+        <v>128</v>
       </c>
       <c r="G268" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H268" s="4" t="inlineStr">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="F269" s="4" t="n">
-        <v>35</v>
+        <v>130</v>
       </c>
       <c r="G269" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H269" s="4" t="inlineStr">
@@ -11583,11 +11583,11 @@
         </is>
       </c>
       <c r="F270" s="4" t="n">
-        <v>21</v>
+        <v>135</v>
       </c>
       <c r="G270" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H270" s="4" t="inlineStr">
@@ -11623,11 +11623,11 @@
         </is>
       </c>
       <c r="F271" s="4" t="n">
-        <v>32</v>
+        <v>118</v>
       </c>
       <c r="G271" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H271" s="4" t="inlineStr">
@@ -11663,11 +11663,11 @@
         </is>
       </c>
       <c r="F272" s="4" t="n">
-        <v>41</v>
+        <v>127</v>
       </c>
       <c r="G272" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H272" s="4" t="inlineStr">
@@ -11703,11 +11703,11 @@
         </is>
       </c>
       <c r="F273" s="4" t="n">
-        <v>39</v>
+        <v>140</v>
       </c>
       <c r="G273" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr">
@@ -11743,11 +11743,11 @@
         </is>
       </c>
       <c r="F274" s="4" t="n">
-        <v>37</v>
+        <v>128</v>
       </c>
       <c r="G274" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H274" s="4" t="inlineStr">
@@ -11783,11 +11783,11 @@
         </is>
       </c>
       <c r="F275" s="4" t="n">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="G275" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr">
@@ -11823,11 +11823,11 @@
         </is>
       </c>
       <c r="F276" s="4" t="n">
-        <v>37</v>
+        <v>142</v>
       </c>
       <c r="G276" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:43</t>
         </is>
       </c>
       <c r="H276" s="4" t="inlineStr">
@@ -11863,11 +11863,11 @@
         </is>
       </c>
       <c r="F277" s="4" t="n">
-        <v>47</v>
+        <v>143</v>
       </c>
       <c r="G277" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr">
@@ -11903,11 +11903,11 @@
         </is>
       </c>
       <c r="F278" s="4" t="n">
-        <v>22</v>
+        <v>127</v>
       </c>
       <c r="G278" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr">
@@ -11943,11 +11943,11 @@
         </is>
       </c>
       <c r="F279" s="4" t="n">
-        <v>21</v>
+        <v>180</v>
       </c>
       <c r="G279" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr">
@@ -11983,11 +11983,11 @@
         </is>
       </c>
       <c r="F280" s="4" t="n">
-        <v>27</v>
+        <v>158</v>
       </c>
       <c r="G280" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H280" s="4" t="inlineStr">
@@ -12023,11 +12023,11 @@
         </is>
       </c>
       <c r="F281" s="4" t="n">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="G281" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr">
@@ -12063,11 +12063,11 @@
         </is>
       </c>
       <c r="F282" s="4" t="n">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="G282" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H282" s="4" t="inlineStr">
@@ -12103,11 +12103,11 @@
         </is>
       </c>
       <c r="F283" s="4" t="n">
-        <v>43</v>
+        <v>139</v>
       </c>
       <c r="G283" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr">
@@ -12143,11 +12143,11 @@
         </is>
       </c>
       <c r="F284" s="4" t="n">
-        <v>47</v>
+        <v>149</v>
       </c>
       <c r="G284" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H284" s="4" t="inlineStr">
@@ -12183,11 +12183,11 @@
         </is>
       </c>
       <c r="F285" s="4" t="n">
-        <v>42</v>
+        <v>148</v>
       </c>
       <c r="G285" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr">
@@ -12223,11 +12223,11 @@
         </is>
       </c>
       <c r="F286" s="4" t="n">
-        <v>16</v>
+        <v>136</v>
       </c>
       <c r="G286" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:44</t>
         </is>
       </c>
       <c r="H286" s="4" t="inlineStr">
@@ -12263,11 +12263,11 @@
         </is>
       </c>
       <c r="F287" s="4" t="n">
-        <v>47</v>
+        <v>144</v>
       </c>
       <c r="G287" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr">
@@ -12303,11 +12303,11 @@
         </is>
       </c>
       <c r="F288" s="4" t="n">
-        <v>24</v>
+        <v>142</v>
       </c>
       <c r="G288" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H288" s="4" t="inlineStr">
@@ -12343,11 +12343,11 @@
         </is>
       </c>
       <c r="F289" s="4" t="n">
-        <v>31</v>
+        <v>169</v>
       </c>
       <c r="G289" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr">
@@ -12383,11 +12383,11 @@
         </is>
       </c>
       <c r="F290" s="4" t="n">
-        <v>20</v>
+        <v>124</v>
       </c>
       <c r="G290" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H290" s="4" t="inlineStr">
@@ -12423,11 +12423,11 @@
         </is>
       </c>
       <c r="F291" s="4" t="n">
-        <v>20</v>
+        <v>147</v>
       </c>
       <c r="G291" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr">
@@ -12463,11 +12463,11 @@
         </is>
       </c>
       <c r="F292" s="4" t="n">
-        <v>18</v>
+        <v>195</v>
       </c>
       <c r="G292" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H292" s="4" t="inlineStr">
@@ -12503,11 +12503,11 @@
         </is>
       </c>
       <c r="F293" s="4" t="n">
-        <v>29</v>
+        <v>245</v>
       </c>
       <c r="G293" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:45</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr">
@@ -12543,11 +12543,11 @@
         </is>
       </c>
       <c r="F294" s="4" t="n">
-        <v>32</v>
+        <v>222</v>
       </c>
       <c r="G294" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:46</t>
         </is>
       </c>
       <c r="H294" s="4" t="inlineStr">
@@ -12583,11 +12583,11 @@
         </is>
       </c>
       <c r="F295" s="4" t="n">
-        <v>46</v>
+        <v>236</v>
       </c>
       <c r="G295" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:46</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr">
@@ -12623,11 +12623,11 @@
         </is>
       </c>
       <c r="F296" s="4" t="n">
-        <v>48</v>
+        <v>170</v>
       </c>
       <c r="G296" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:46</t>
         </is>
       </c>
       <c r="H296" s="4" t="inlineStr">
@@ -12663,11 +12663,11 @@
         </is>
       </c>
       <c r="F297" s="4" t="n">
-        <v>30</v>
+        <v>246</v>
       </c>
       <c r="G297" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:46</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr">
@@ -12703,11 +12703,11 @@
         </is>
       </c>
       <c r="F298" s="4" t="n">
-        <v>20</v>
+        <v>175</v>
       </c>
       <c r="G298" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:46</t>
         </is>
       </c>
       <c r="H298" s="4" t="inlineStr">
@@ -12743,11 +12743,11 @@
         </is>
       </c>
       <c r="F299" s="4" t="n">
-        <v>33</v>
+        <v>194</v>
       </c>
       <c r="G299" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:47</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr">
@@ -12783,11 +12783,11 @@
         </is>
       </c>
       <c r="F300" s="4" t="n">
-        <v>22</v>
+        <v>126</v>
       </c>
       <c r="G300" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:47</t>
         </is>
       </c>
       <c r="H300" s="4" t="inlineStr">
@@ -12823,11 +12823,11 @@
         </is>
       </c>
       <c r="F301" s="4" t="n">
-        <v>17</v>
+        <v>145</v>
       </c>
       <c r="G301" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29 02:38:24</t>
+          <t>2026-07-29 02:41:47</t>
         </is>
       </c>
       <c r="H301" s="4" t="inlineStr">

</xml_diff>